<commit_message>
Add schema_data vertical-merge case, row grouping, and raw_data goldens.
Set is_row_grouped from single-column multi-row data merges; add readRawData with TestReadRawDataSchemaData fixtures for each data-band case.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/excel/testdata/schema_data/schema_data_tests.xlsx
+++ b/excel/testdata/schema_data/schema_data_tests.xlsx
@@ -11,6 +11,7 @@
     <sheet name="data-empty-column" sheetId="2" r:id="rId5"/>
     <sheet name="data-empty-cell" sheetId="3" r:id="rId6"/>
     <sheet name="data-mixed-types" sheetId="4" r:id="rId7"/>
+    <sheet name="data-vertical-merge" sheetId="5" r:id="rId8"/>
   </sheets>
   <calcPr calcId="122211"/>
 </workbook>
@@ -584,4 +585,57 @@
     </row>
   </sheetData>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2"/>
+      <c r="B3" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:A3"/>
+  </mergeCells>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Reject multi-column merges in the data band and extend schema_data fixtures.
Add data-formula and data-horizontal-merge cases; horizontal data merge errors like leaf-header policy. Document schema_data initial pass complete.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/excel/testdata/schema_data/schema_data_tests.xlsx
+++ b/excel/testdata/schema_data/schema_data_tests.xlsx
@@ -12,6 +12,8 @@
     <sheet name="data-empty-cell" sheetId="3" r:id="rId6"/>
     <sheet name="data-mixed-types" sheetId="4" r:id="rId7"/>
     <sheet name="data-vertical-merge" sheetId="5" r:id="rId8"/>
+    <sheet name="data-horizontal-merge" sheetId="6" r:id="rId9"/>
+    <sheet name="data-formula" sheetId="7" r:id="rId10"/>
   </sheets>
   <calcPr calcId="122211"/>
 </workbook>
@@ -638,4 +640,110 @@
     <mergeCell ref="A2:A3"/>
   </mergeCells>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="2"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B2:C2"/>
+  </mergeCells>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="2" t="str">
+        <f>B2&amp;"-calc"</f>
+        <v>7</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add schema_data fixtures for multi-group vertical merges.
Exercise 12-row bands with 6×2 and 3×4 row grouping on A/B and B/C columns.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/excel/testdata/schema_data/schema_data_tests.xlsx
+++ b/excel/testdata/schema_data/schema_data_tests.xlsx
@@ -12,15 +12,17 @@
     <sheet name="data-empty-cell" sheetId="3" r:id="rId6"/>
     <sheet name="data-mixed-types" sheetId="4" r:id="rId7"/>
     <sheet name="data-vertical-merge" sheetId="5" r:id="rId8"/>
-    <sheet name="data-horizontal-merge" sheetId="6" r:id="rId9"/>
-    <sheet name="data-formula" sheetId="7" r:id="rId10"/>
+    <sheet name="data-vmerge-a6-b3" sheetId="6" r:id="rId9"/>
+    <sheet name="data-vmerge-b6-c3" sheetId="7" r:id="rId10"/>
+    <sheet name="data-horizontal-merge" sheetId="8" r:id="rId11"/>
+    <sheet name="data-formula" sheetId="9" r:id="rId12"/>
   </sheets>
   <calcPr calcId="122211"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="39">
   <si>
     <t>headerA</t>
   </si>
@@ -56,6 +58,87 @@
   </si>
   <si>
     <t>r4cC</t>
+  </si>
+  <si>
+    <t>r5cA</t>
+  </si>
+  <si>
+    <t>r6cA</t>
+  </si>
+  <si>
+    <t>r7cA</t>
+  </si>
+  <si>
+    <t>r8cA</t>
+  </si>
+  <si>
+    <t>r9cA</t>
+  </si>
+  <si>
+    <t>r10cA</t>
+  </si>
+  <si>
+    <t>r11cA</t>
+  </si>
+  <si>
+    <t>r12cA</t>
+  </si>
+  <si>
+    <t>r13cA</t>
+  </si>
+  <si>
+    <t>r5cB</t>
+  </si>
+  <si>
+    <t>r6cB</t>
+  </si>
+  <si>
+    <t>r7cB</t>
+  </si>
+  <si>
+    <t>r8cB</t>
+  </si>
+  <si>
+    <t>r9cB</t>
+  </si>
+  <si>
+    <t>r10cB</t>
+  </si>
+  <si>
+    <t>r11cB</t>
+  </si>
+  <si>
+    <t>r12cB</t>
+  </si>
+  <si>
+    <t>r13cB</t>
+  </si>
+  <si>
+    <t>r5cC</t>
+  </si>
+  <si>
+    <t>r6cC</t>
+  </si>
+  <si>
+    <t>r7cC</t>
+  </si>
+  <si>
+    <t>r8cC</t>
+  </si>
+  <si>
+    <t>r9cC</t>
+  </si>
+  <si>
+    <t>r10cC</t>
+  </si>
+  <si>
+    <t>r11cC</t>
+  </si>
+  <si>
+    <t>r12cC</t>
+  </si>
+  <si>
+    <t>r13cC</t>
   </si>
 </sst>
 </file>
@@ -664,33 +747,103 @@
       <c r="B2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="2"/>
+      <c r="C2" s="2" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>7</v>
-      </c>
+      <c r="A3" s="2"/>
+      <c r="B3" s="2"/>
       <c r="C3" s="2" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>8</v>
-      </c>
+      <c r="A4" s="2"/>
+      <c r="B4" s="2"/>
       <c r="C4" s="2" t="s">
         <v>11</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="2"/>
+      <c r="B5" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2"/>
+      <c r="B6" s="2"/>
+      <c r="C6" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2"/>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2"/>
+      <c r="B9" s="2"/>
+      <c r="C9" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2"/>
+      <c r="B10" s="2"/>
+      <c r="C10" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2"/>
+      <c r="B11" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2"/>
+      <c r="B12" s="2"/>
+      <c r="C12" s="2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2"/>
+      <c r="B13" s="2"/>
+      <c r="C13" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="B2:C2"/>
+  <mergeCells count="6">
+    <mergeCell ref="A2:A7"/>
+    <mergeCell ref="A8:A13"/>
+    <mergeCell ref="B2:B4"/>
+    <mergeCell ref="B5:B7"/>
+    <mergeCell ref="B8:B10"/>
+    <mergeCell ref="B11:B13"/>
   </mergeCells>
 </worksheet>
 </file>
@@ -725,6 +878,182 @@
       <c r="A3" s="2" t="s">
         <v>4</v>
       </c>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="2"/>
+      <c r="C4" s="2"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" s="2"/>
+      <c r="C6" s="2"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" s="2"/>
+      <c r="C9" s="2"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B10" s="2"/>
+      <c r="C10" s="2"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B11" s="2"/>
+      <c r="C11" s="2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B12" s="2"/>
+      <c r="C12" s="2"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B13" s="2"/>
+      <c r="C13" s="2"/>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="B2:B7"/>
+    <mergeCell ref="B8:B13"/>
+    <mergeCell ref="C2:C4"/>
+    <mergeCell ref="C5:C7"/>
+    <mergeCell ref="C8:C10"/>
+    <mergeCell ref="C11:C13"/>
+  </mergeCells>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="2"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B2:C2"/>
+  </mergeCells>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="s">
+        <v>4</v>
+      </c>
       <c r="B3" s="2" t="str">
         <f>B2&amp;"-calc"</f>
         <v>7</v>

</xml_diff>